<commit_message>
Introduction of Member Fixtures and General bug-fixes
</commit_message>
<xml_diff>
--- a/Supabase Configuration/member_import2.xlsx
+++ b/Supabase Configuration/member_import2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\bowls_saas\Supabase Configuration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D1EC68B-4DF8-4631-B133-FC742DC09BDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF065BEC-4B3F-460A-821D-D44D789BCFE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="348" yWindow="336" windowWidth="22458" windowHeight="13092" xr2:uid="{8E3A18D9-674A-4ACB-9EC6-C6F5A6D51734}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{8E3A18D9-674A-4ACB-9EC6-C6F5A6D51734}"/>
   </bookViews>
   <sheets>
     <sheet name="member_import" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="35">
   <si>
     <t>password</t>
   </si>
@@ -96,6 +96,48 @@
   </si>
   <si>
     <t>rodrigues</t>
+  </si>
+  <si>
+    <t>dave</t>
+  </si>
+  <si>
+    <t>curtis</t>
+  </si>
+  <si>
+    <t>julie</t>
+  </si>
+  <si>
+    <t>tullett</t>
+  </si>
+  <si>
+    <t>andrea</t>
+  </si>
+  <si>
+    <t>jebb</t>
+  </si>
+  <si>
+    <t>bob</t>
+  </si>
+  <si>
+    <t>parker</t>
+  </si>
+  <si>
+    <t>ian</t>
+  </si>
+  <si>
+    <t>remedios</t>
+  </si>
+  <si>
+    <t>hill</t>
+  </si>
+  <si>
+    <t>carol</t>
+  </si>
+  <si>
+    <t>sullivan</t>
+  </si>
+  <si>
+    <t>susan</t>
   </si>
 </sst>
 </file>
@@ -956,7 +998,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{080DD124-4D3D-4E29-B146-0C9CEB45B0AF}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="3" max="3" width="26.5234375" bestFit="1" customWidth="1"/>
@@ -984,7 +1026,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="str">
-        <f>A2&amp;"."&amp;B2&amp;"@lcpibc.co.uk"</f>
+        <f t="shared" ref="C2:C18" si="0">A2&amp;"."&amp;B2&amp;"@lcpibc.co.uk"</f>
         <v>tony.alicock@lcpibc.co.uk</v>
       </c>
       <c r="D2" t="str">
@@ -1000,7 +1042,7 @@
         <v>4</v>
       </c>
       <c r="C3" t="str">
-        <f>A3&amp;"."&amp;B3&amp;"@lcpibc.co.uk"</f>
+        <f t="shared" si="0"/>
         <v>lynn.dempsey@lcpibc.co.uk</v>
       </c>
       <c r="D3" t="str">
@@ -1016,7 +1058,7 @@
         <v>8</v>
       </c>
       <c r="C4" t="str">
-        <f>A4&amp;"."&amp;B4&amp;"@lcpibc.co.uk"</f>
+        <f t="shared" si="0"/>
         <v>kay.gordon@lcpibc.co.uk</v>
       </c>
       <c r="D4" t="str">
@@ -1032,7 +1074,7 @@
         <v>11</v>
       </c>
       <c r="C5" t="str">
-        <f>A5&amp;"."&amp;B5&amp;"@lcpibc.co.uk"</f>
+        <f t="shared" si="0"/>
         <v>clive.edgehill@lcpibc.co.uk</v>
       </c>
       <c r="D5" t="str">
@@ -1048,7 +1090,7 @@
         <v>12</v>
       </c>
       <c r="C6" t="str">
-        <f>A6&amp;"."&amp;B6&amp;"@lcpibc.co.uk"</f>
+        <f t="shared" si="0"/>
         <v>tony.hodge@lcpibc.co.uk</v>
       </c>
       <c r="D6" t="str">
@@ -1064,11 +1106,11 @@
         <v>13</v>
       </c>
       <c r="C7" t="str">
-        <f>A7&amp;"."&amp;B7&amp;"@lcpibc.co.uk"</f>
+        <f t="shared" si="0"/>
         <v>kay.lanston@lcpibc.co.uk</v>
       </c>
       <c r="D7" t="str">
-        <f t="shared" ref="D7:D11" si="0">"password"</f>
+        <f t="shared" ref="D7:D11" si="1">"password"</f>
         <v>password</v>
       </c>
     </row>
@@ -1080,11 +1122,11 @@
         <v>15</v>
       </c>
       <c r="C8" t="str">
-        <f>A8&amp;"."&amp;B8&amp;"@lcpibc.co.uk"</f>
+        <f t="shared" si="0"/>
         <v>phil.lennon@lcpibc.co.uk</v>
       </c>
       <c r="D8" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>password</v>
       </c>
     </row>
@@ -1096,11 +1138,11 @@
         <v>17</v>
       </c>
       <c r="C9" t="str">
-        <f>A9&amp;"."&amp;B9&amp;"@lcpibc.co.uk"</f>
+        <f t="shared" si="0"/>
         <v>terry.moore@lcpibc.co.uk</v>
       </c>
       <c r="D9" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>password</v>
       </c>
     </row>
@@ -1112,11 +1154,11 @@
         <v>17</v>
       </c>
       <c r="C10" t="str">
-        <f>A10&amp;"."&amp;B10&amp;"@lcpibc.co.uk"</f>
+        <f t="shared" si="0"/>
         <v>sue.moore@lcpibc.co.uk</v>
       </c>
       <c r="D10" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>password</v>
       </c>
     </row>
@@ -1128,12 +1170,117 @@
         <v>20</v>
       </c>
       <c r="C11" t="str">
-        <f>A11&amp;"."&amp;B11&amp;"@lcpibc.co.uk"</f>
+        <f t="shared" si="0"/>
         <v>tracey.rodrigues@lcpibc.co.uk</v>
       </c>
       <c r="D11" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>password</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" t="str">
+        <f t="shared" si="0"/>
+        <v>dave.curtis@lcpibc.co.uk</v>
+      </c>
+      <c r="D12" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" t="str">
+        <f t="shared" si="0"/>
+        <v>julie.tullett@lcpibc.co.uk</v>
+      </c>
+      <c r="D13" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" t="str">
+        <f t="shared" si="0"/>
+        <v>andrea.jebb@lcpibc.co.uk</v>
+      </c>
+      <c r="D14" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="str">
+        <f t="shared" si="0"/>
+        <v>bob.parker@lcpibc.co.uk</v>
+      </c>
+      <c r="D15" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="0"/>
+        <v>ian.remedios@lcpibc.co.uk</v>
+      </c>
+      <c r="D16" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" t="str">
+        <f t="shared" si="0"/>
+        <v>susan.hill@lcpibc.co.uk</v>
+      </c>
+      <c r="D17" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" t="str">
+        <f t="shared" si="0"/>
+        <v>carol.sullivan@lcpibc.co.uk</v>
+      </c>
+      <c r="D18" t="s">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>